<commit_message>
Fix: change color on tkinter
</commit_message>
<xml_diff>
--- a/Student_analysis_35.0.xlsx
+++ b/Student_analysis_35.0.xlsx
@@ -449,7 +449,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Numbers</t>
+          <t>Safety and Tools</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -457,7 +457,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Exceeding Expectation</t>
+          <t>Meeting Expectation</t>
         </is>
       </c>
     </row>
@@ -468,7 +468,7 @@
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Algebra</t>
+          <t>Technical Drawing</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -487,7 +487,7 @@
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Measurement</t>
+          <t>Material and Production</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -495,7 +495,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Exceeding Expectation</t>
+          <t>Approaching Expectation</t>
         </is>
       </c>
     </row>
@@ -506,7 +506,7 @@
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Geomentry</t>
+          <t>Electricity and Electronics</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -514,7 +514,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Exceeding Expectation</t>
+          <t>Below Expectation</t>
         </is>
       </c>
     </row>
@@ -525,7 +525,7 @@
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Data Handling and Probability</t>
+          <t>Computer Studies and Digital Literacy</t>
         </is>
       </c>
       <c r="D6" t="n">

</xml_diff>